<commit_message>
Deploying to gh-pages from @ codeforIATI/codelists@6498964892ddc7d3455b1156239b0d1dd3dc3550 🚀
</commit_message>
<xml_diff>
--- a/api/1/clv1/codelist/ReportingOrganisation.xlsx
+++ b/api/1/clv1/codelist/ReportingOrganisation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6415" uniqueCount="4253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6502" uniqueCount="4311">
   <si>
     <t>code</t>
   </si>
@@ -364,7 +364,7 @@
     <t>GB-SC-SC030289</t>
   </si>
   <si>
-    <t>Mercy Corps Europe</t>
+    <t>Prosper Global (UK)</t>
   </si>
   <si>
     <t>GB-COH-1100897</t>
@@ -2617,7 +2617,7 @@
     <t>mz-moj-64vq1</t>
   </si>
   <si>
-    <t>Ajuda de Desenvolvimento de Povo para Povo (ADPP)</t>
+    <t>Ajuda de Desenvolvimento de Povo para Povo (Mozambique)</t>
   </si>
   <si>
     <t>GB-COH-2394229</t>
@@ -2683,7 +2683,7 @@
     <t>GB-COH-00986729</t>
   </si>
   <si>
-    <t>Natural Resources Institute, University of Greenwich.</t>
+    <t>London and South East University Group (LASE)</t>
   </si>
   <si>
     <t>NL-KVK-41215393</t>
@@ -4615,7 +4615,7 @@
     <t>BE-BCE_KBO-0413986102</t>
   </si>
   <si>
-    <t>Wereldsolidariteit-Solidarité Mondiale (WSM)</t>
+    <t>WSM</t>
   </si>
   <si>
     <t>NG-CAC-692943</t>
@@ -6409,7 +6409,7 @@
     <t>US-EIN-91-1148123</t>
   </si>
   <si>
-    <t>Mercy Corps Global</t>
+    <t>Prosper Global (US)</t>
   </si>
   <si>
     <t>GB-CHC-1108718</t>
@@ -6433,7 +6433,7 @@
     <t>NL-KVK-70333564</t>
   </si>
   <si>
-    <t>Mercy Corps Netherlands</t>
+    <t>Prosper Global (NL)</t>
   </si>
   <si>
     <t>PE-SUNARP-12623829</t>
@@ -9370,6 +9370,12 @@
     <t>Burundi Leadership Training Programme</t>
   </si>
   <si>
+    <t>KE-RCO-CPR201020397</t>
+  </si>
+  <si>
+    <t>InformAction</t>
+  </si>
+  <si>
     <t>FI-PRO3087706-5</t>
   </si>
   <si>
@@ -12508,6 +12514,48 @@
     <t>Institute for Fiscal Studies</t>
   </si>
   <si>
+    <t>SE-ON-802415-4737</t>
+  </si>
+  <si>
+    <t>SWEDWATCH</t>
+  </si>
+  <si>
+    <t>UG-RSB-80020002460437</t>
+  </si>
+  <si>
+    <t>Emata</t>
+  </si>
+  <si>
+    <t>TZ-NNCB-00NGO-RI-00199</t>
+  </si>
+  <si>
+    <t>THE CENTRE FOR COUNSELLING, NUTRITION AND HEALTH CARE</t>
+  </si>
+  <si>
+    <t>PH-SEC-CN200718575</t>
+  </si>
+  <si>
+    <t>National Union of Peoples' Lawyers</t>
+  </si>
+  <si>
+    <t>XI-ROR-03r8z3t63</t>
+  </si>
+  <si>
+    <t>University of NSW</t>
+  </si>
+  <si>
+    <t>IN-MCA-U74999TN2010PTC076608</t>
+  </si>
+  <si>
+    <t>Athena Infonomics India Private Limited</t>
+  </si>
+  <si>
+    <t>CH-FDJP-CHE114952278</t>
+  </si>
+  <si>
+    <t>Summit Alliances International</t>
+  </si>
+  <si>
     <t>MM-MHA-0004-1951</t>
   </si>
   <si>
@@ -12550,6 +12598,12 @@
     <t>Action For Sustainability Initiative</t>
   </si>
   <si>
+    <t>TZ-NNCB-00NGOR200060</t>
+  </si>
+  <si>
+    <t>KIMAS(KITOVU CHA MAENDELEO SAFI)</t>
+  </si>
+  <si>
     <t>KE-NCB-218051200902226007</t>
   </si>
   <si>
@@ -12568,6 +12622,30 @@
     <t>Integrated Research and Action For Developement</t>
   </si>
   <si>
+    <t>MW-NBM-L23038</t>
+  </si>
+  <si>
+    <t>Global Health Informatics Institute</t>
+  </si>
+  <si>
+    <t>XI-ROR-00nzqgm49</t>
+  </si>
+  <si>
+    <t>Université Catholique de l'Afrique de l'Ouest _Unité Universitaire à Bobo-Dioulasso (UCAO-UUB)</t>
+  </si>
+  <si>
+    <t>IQ-NGO-1H1803026</t>
+  </si>
+  <si>
+    <t>Kurdistan Organization for Human Rights Watch</t>
+  </si>
+  <si>
+    <t>SE-ON-202100-6420</t>
+  </si>
+  <si>
+    <t>Swedish Agency for Marine and Water Management</t>
+  </si>
+  <si>
     <t>GH-TIN-V0004994299</t>
   </si>
   <si>
@@ -12586,24 +12664,102 @@
     <t>Chiang Mai University</t>
   </si>
   <si>
+    <t>SE-ON-802007-5290</t>
+  </si>
+  <si>
+    <t>International Council of Swedish Industry, NIR</t>
+  </si>
+  <si>
+    <t>TZ-NNCB-00NGOR0266</t>
+  </si>
+  <si>
+    <t>Inland Development Services</t>
+  </si>
+  <si>
+    <t>ZM-RS-10235225</t>
+  </si>
+  <si>
+    <t>Zambia Council for Social Development (ZCSD)</t>
+  </si>
+  <si>
     <t>GB-UKPRN-10004180</t>
   </si>
   <si>
     <t>Manchester Metropolitan University</t>
   </si>
   <si>
+    <t>XI-ROR-0130VHY65</t>
+  </si>
+  <si>
+    <t>Biomedical Research and Training Institute</t>
+  </si>
+  <si>
     <t>CH-FDJP-CHE-207616410</t>
   </si>
   <si>
     <t>Centre on Armed Groups</t>
   </si>
   <si>
+    <t>TZ-NNCB-00NGO-08231</t>
+  </si>
+  <si>
+    <t>Foundation for Local Capacity in Agricultural Development</t>
+  </si>
+  <si>
+    <t>TZ-NNCB-OONGO-R-7428</t>
+  </si>
+  <si>
+    <t>Chamwiilee Agro-Live</t>
+  </si>
+  <si>
+    <t>TZ-NNCB-00NGOR7295</t>
+  </si>
+  <si>
+    <t>MAZINGIRA NI UHAI (mnu)</t>
+  </si>
+  <si>
+    <t>GW-NIF-910000069</t>
+  </si>
+  <si>
+    <t>Ajuda de Desenvolvimento de Povo para Povo (Guinea-Bissau)</t>
+  </si>
+  <si>
+    <t>IN-PAN-AAATN2786N</t>
+  </si>
+  <si>
+    <t>Nightingales Medical Trust</t>
+  </si>
+  <si>
+    <t>XI-ROR-05e15a779</t>
+  </si>
+  <si>
+    <t>All India Institute of Medical Sciences Jodhpur</t>
+  </si>
+  <si>
+    <t>TZ-NNCB-00NGO00010158</t>
+  </si>
+  <si>
+    <t>CIVIC SOCIAL PROTECTION FOUNDATION (CSP)</t>
+  </si>
+  <si>
+    <t>GB-COH-17211046</t>
+  </si>
+  <si>
+    <t>SGE Commission</t>
+  </si>
+  <si>
     <t>GB-CHC-1193984</t>
   </si>
   <si>
     <t>Vodafone Foundation</t>
   </si>
   <si>
+    <t>VN-TIN-0101088071</t>
+  </si>
+  <si>
+    <t>Hanoi University of Public Health</t>
+  </si>
+  <si>
     <t>GB-UKPRN-10007800</t>
   </si>
   <si>
@@ -12622,6 +12778,12 @@
     <t>Borneo Nature Foundation</t>
   </si>
   <si>
+    <t>SE-ON-802407-6419</t>
+  </si>
+  <si>
+    <t>Swedish International Liberal Centre</t>
+  </si>
+  <si>
     <t>SE-ON-802001-6047</t>
   </si>
   <si>
@@ -12646,6 +12808,12 @@
     <t>SOS Children's Villages Ukraine</t>
   </si>
   <si>
+    <t>TZ-NNCB-00NGO0008958</t>
+  </si>
+  <si>
+    <t>Smart Farmers and Transformation (SFT)</t>
+  </si>
+  <si>
     <t>XI-ROR-026A3NK20</t>
   </si>
   <si>
@@ -12680,6 +12848,12 @@
   </si>
   <si>
     <t>Unión de Afectados y Afectadas por las Operaciones Petroleras de Texaco – UDAPT</t>
+  </si>
+  <si>
+    <t>ZA-NPO-255-261</t>
+  </si>
+  <si>
+    <t>Open Cities Lab NPC</t>
   </si>
   <si>
     <t>SE-ON-802467-0195</t>
@@ -13104,7 +13278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2137"/>
+  <dimension ref="A1:G2166"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -30768,7 +30942,7 @@
         <v>3194</v>
       </c>
       <c r="B1605" t="s">
-        <v>2295</v>
+        <v>3195</v>
       </c>
       <c r="D1605" t="s">
         <v>9</v>
@@ -30776,10 +30950,10 @@
     </row>
     <row r="1606" spans="1:4">
       <c r="A1606" t="s">
-        <v>3195</v>
+        <v>3196</v>
       </c>
       <c r="B1606" t="s">
-        <v>3196</v>
+        <v>2295</v>
       </c>
       <c r="D1606" t="s">
         <v>9</v>
@@ -31010,7 +31184,7 @@
         <v>3237</v>
       </c>
       <c r="B1627" t="s">
-        <v>3228</v>
+        <v>3238</v>
       </c>
       <c r="D1627" t="s">
         <v>9</v>
@@ -31018,10 +31192,10 @@
     </row>
     <row r="1628" spans="1:4">
       <c r="A1628" t="s">
-        <v>3238</v>
+        <v>3239</v>
       </c>
       <c r="B1628" t="s">
-        <v>3239</v>
+        <v>3230</v>
       </c>
       <c r="D1628" t="s">
         <v>9</v>
@@ -34134,7 +34308,7 @@
         <v>3804</v>
       </c>
       <c r="B1911" t="s">
-        <v>2673</v>
+        <v>3805</v>
       </c>
       <c r="D1911" t="s">
         <v>9</v>
@@ -34142,10 +34316,10 @@
     </row>
     <row r="1912" spans="1:4">
       <c r="A1912" t="s">
-        <v>3805</v>
+        <v>3806</v>
       </c>
       <c r="B1912" t="s">
-        <v>3806</v>
+        <v>2673</v>
       </c>
       <c r="D1912" t="s">
         <v>9</v>
@@ -34167,7 +34341,7 @@
         <v>3809</v>
       </c>
       <c r="B1914" t="s">
-        <v>3198</v>
+        <v>3810</v>
       </c>
       <c r="D1914" t="s">
         <v>9</v>
@@ -34175,10 +34349,10 @@
     </row>
     <row r="1915" spans="1:4">
       <c r="A1915" t="s">
-        <v>3810</v>
+        <v>3811</v>
       </c>
       <c r="B1915" t="s">
-        <v>3811</v>
+        <v>3200</v>
       </c>
       <c r="D1915" t="s">
         <v>9</v>
@@ -35289,7 +35463,7 @@
         <v>4012</v>
       </c>
       <c r="B2016" t="s">
-        <v>2171</v>
+        <v>4013</v>
       </c>
       <c r="D2016" t="s">
         <v>9</v>
@@ -35297,10 +35471,10 @@
     </row>
     <row r="2017" spans="1:4">
       <c r="A2017" t="s">
-        <v>4013</v>
+        <v>4014</v>
       </c>
       <c r="B2017" t="s">
-        <v>4014</v>
+        <v>2171</v>
       </c>
       <c r="D2017" t="s">
         <v>9</v>
@@ -36070,7 +36244,7 @@
         <v>4153</v>
       </c>
       <c r="B2087" t="s">
-        <v>2888</v>
+        <v>4154</v>
       </c>
       <c r="D2087" t="s">
         <v>9</v>
@@ -36078,10 +36252,10 @@
     </row>
     <row r="2088" spans="1:4">
       <c r="A2088" t="s">
-        <v>4154</v>
+        <v>4155</v>
       </c>
       <c r="B2088" t="s">
-        <v>4155</v>
+        <v>2888</v>
       </c>
       <c r="D2088" t="s">
         <v>9</v>
@@ -36609,7 +36783,7 @@
         <v>4250</v>
       </c>
       <c r="B2136" t="s">
-        <v>3283</v>
+        <v>4251</v>
       </c>
       <c r="D2136" t="s">
         <v>9</v>
@@ -36617,12 +36791,331 @@
     </row>
     <row r="2137" spans="1:4">
       <c r="A2137" t="s">
-        <v>4251</v>
+        <v>4252</v>
       </c>
       <c r="B2137" t="s">
-        <v>4252</v>
+        <v>4253</v>
       </c>
       <c r="D2137" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2138" spans="1:4">
+      <c r="A2138" t="s">
+        <v>4254</v>
+      </c>
+      <c r="B2138" t="s">
+        <v>4255</v>
+      </c>
+      <c r="D2138" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2139" spans="1:4">
+      <c r="A2139" t="s">
+        <v>4256</v>
+      </c>
+      <c r="B2139" t="s">
+        <v>4257</v>
+      </c>
+      <c r="D2139" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2140" spans="1:4">
+      <c r="A2140" t="s">
+        <v>4258</v>
+      </c>
+      <c r="B2140" t="s">
+        <v>4259</v>
+      </c>
+      <c r="D2140" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2141" spans="1:4">
+      <c r="A2141" t="s">
+        <v>4260</v>
+      </c>
+      <c r="B2141" t="s">
+        <v>4261</v>
+      </c>
+      <c r="D2141" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2142" spans="1:4">
+      <c r="A2142" t="s">
+        <v>4262</v>
+      </c>
+      <c r="B2142" t="s">
+        <v>4263</v>
+      </c>
+      <c r="D2142" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2143" spans="1:4">
+      <c r="A2143" t="s">
+        <v>4264</v>
+      </c>
+      <c r="B2143" t="s">
+        <v>4265</v>
+      </c>
+      <c r="D2143" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2144" spans="1:4">
+      <c r="A2144" t="s">
+        <v>4266</v>
+      </c>
+      <c r="B2144" t="s">
+        <v>4267</v>
+      </c>
+      <c r="D2144" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2145" spans="1:4">
+      <c r="A2145" t="s">
+        <v>4268</v>
+      </c>
+      <c r="B2145" t="s">
+        <v>4269</v>
+      </c>
+      <c r="D2145" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2146" spans="1:4">
+      <c r="A2146" t="s">
+        <v>4270</v>
+      </c>
+      <c r="B2146" t="s">
+        <v>4271</v>
+      </c>
+      <c r="D2146" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2147" spans="1:4">
+      <c r="A2147" t="s">
+        <v>4272</v>
+      </c>
+      <c r="B2147" t="s">
+        <v>4273</v>
+      </c>
+      <c r="D2147" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2148" spans="1:4">
+      <c r="A2148" t="s">
+        <v>4274</v>
+      </c>
+      <c r="B2148" t="s">
+        <v>4275</v>
+      </c>
+      <c r="D2148" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2149" spans="1:4">
+      <c r="A2149" t="s">
+        <v>4276</v>
+      </c>
+      <c r="B2149" t="s">
+        <v>4277</v>
+      </c>
+      <c r="D2149" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2150" spans="1:4">
+      <c r="A2150" t="s">
+        <v>4278</v>
+      </c>
+      <c r="B2150" t="s">
+        <v>4279</v>
+      </c>
+      <c r="D2150" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2151" spans="1:4">
+      <c r="A2151" t="s">
+        <v>4280</v>
+      </c>
+      <c r="B2151" t="s">
+        <v>4281</v>
+      </c>
+      <c r="D2151" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2152" spans="1:4">
+      <c r="A2152" t="s">
+        <v>4282</v>
+      </c>
+      <c r="B2152" t="s">
+        <v>4283</v>
+      </c>
+      <c r="D2152" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2153" spans="1:4">
+      <c r="A2153" t="s">
+        <v>4284</v>
+      </c>
+      <c r="B2153" t="s">
+        <v>4285</v>
+      </c>
+      <c r="D2153" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2154" spans="1:4">
+      <c r="A2154" t="s">
+        <v>4286</v>
+      </c>
+      <c r="B2154" t="s">
+        <v>4287</v>
+      </c>
+      <c r="D2154" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2155" spans="1:4">
+      <c r="A2155" t="s">
+        <v>4288</v>
+      </c>
+      <c r="B2155" t="s">
+        <v>4289</v>
+      </c>
+      <c r="D2155" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2156" spans="1:4">
+      <c r="A2156" t="s">
+        <v>4290</v>
+      </c>
+      <c r="B2156" t="s">
+        <v>4291</v>
+      </c>
+      <c r="D2156" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2157" spans="1:4">
+      <c r="A2157" t="s">
+        <v>4292</v>
+      </c>
+      <c r="B2157" t="s">
+        <v>4293</v>
+      </c>
+      <c r="D2157" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2158" spans="1:4">
+      <c r="A2158" t="s">
+        <v>4294</v>
+      </c>
+      <c r="B2158" t="s">
+        <v>4295</v>
+      </c>
+      <c r="D2158" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2159" spans="1:4">
+      <c r="A2159" t="s">
+        <v>4296</v>
+      </c>
+      <c r="B2159" t="s">
+        <v>4297</v>
+      </c>
+      <c r="D2159" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2160" spans="1:4">
+      <c r="A2160" t="s">
+        <v>4298</v>
+      </c>
+      <c r="B2160" t="s">
+        <v>4299</v>
+      </c>
+      <c r="D2160" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2161" spans="1:4">
+      <c r="A2161" t="s">
+        <v>4300</v>
+      </c>
+      <c r="B2161" t="s">
+        <v>4301</v>
+      </c>
+      <c r="D2161" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2162" spans="1:4">
+      <c r="A2162" t="s">
+        <v>4302</v>
+      </c>
+      <c r="B2162" t="s">
+        <v>4303</v>
+      </c>
+      <c r="D2162" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2163" spans="1:4">
+      <c r="A2163" t="s">
+        <v>4304</v>
+      </c>
+      <c r="B2163" t="s">
+        <v>4305</v>
+      </c>
+      <c r="D2163" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2164" spans="1:4">
+      <c r="A2164" t="s">
+        <v>4306</v>
+      </c>
+      <c r="B2164" t="s">
+        <v>4307</v>
+      </c>
+      <c r="D2164" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2165" spans="1:4">
+      <c r="A2165" t="s">
+        <v>4308</v>
+      </c>
+      <c r="B2165" t="s">
+        <v>3285</v>
+      </c>
+      <c r="D2165" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2166" spans="1:4">
+      <c r="A2166" t="s">
+        <v>4309</v>
+      </c>
+      <c r="B2166" t="s">
+        <v>4310</v>
+      </c>
+      <c r="D2166" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>